<commit_message>
Report UX fixes: % instead of 'f.b.', colored title banner, plan-line on trend
- Deviation shown as % (not 'f.b.') in toolbar and landing page
- Report title now on a colored (blue gradient) banner
- trendLine() draws the planned line as blue dotted points when trend rows
  carry a 'plan' value; PackagesTrend Excel sheet gains an optional 'plan' column

Note: only presentation/capability changes — no project data was altered.
</commit_message>
<xml_diff>
--- a/cities/qervend/source.xlsx
+++ b/cities/qervend/source.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="172">
   <si>
     <t>Sahə</t>
   </si>
@@ -1697,21 +1697,24 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="1" max="3" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>80</v>
       </c>
@@ -1719,7 +1722,7 @@
         <v>26.05</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -1727,7 +1730,7 @@
         <v>31.08</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Report fixes (scoped): 3-week Ümumi trend, detailed work-stages, compact title bar, desktop PDF
- Ümumi İcra trendi: 3 real weekly snapshots (28.05, 04.06, 11.06) with plan
  (blue) + actual (red), Ümumi only — from the weekly reports
- Görülən işlər: detailed per-stage view (Qaba işlər, Dam örtüyü, Daxili bəzək,
  MEP, Xarici bəzək, Təsərrüfat) per packet, each = average of the 4 house
  types' Primavera %; with plan vs actual so lag is visible
- Finish date: drop the unsourced 05.11.2026 (it was from the old 23.04 Excel,
  not Primavera). Use Primavera baseline: 30.11.2026, 415 gün
- PDF + Excel buttons moved onto the report-title line (compact)
- PDF: render at desktop width even on mobile, single continuous page (no cuts)
- Responsive layout for mobile (grids/KPIs stack); app: usage hint

Only these parts changed; other data/sections untouched.
</commit_message>
<xml_diff>
--- a/cities/qervend/source.xlsx
+++ b/cities/qervend/source.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="144">
   <si>
     <t>Sahə</t>
   </si>
@@ -75,15 +75,12 @@
     <t>plannedFinish</t>
   </si>
   <si>
-    <t>05.11.2026</t>
+    <t>30.11.2026</t>
   </si>
   <si>
     <t>revisedFinish</t>
   </si>
   <si>
-    <t>30.11.2026</t>
-  </si>
-  <si>
     <t>baselineDays</t>
   </si>
   <si>
@@ -249,7 +246,10 @@
     <t>date</t>
   </si>
   <si>
-    <t>21.05.2026</t>
+    <t>28.05.2026</t>
+  </si>
+  <si>
+    <t>04.06.2026</t>
   </si>
   <si>
     <t>lot_id</t>
@@ -270,42 +270,48 @@
     <t>Cəmi (851 ev)</t>
   </si>
   <si>
+    <t>Qaba işlər</t>
+  </si>
+  <si>
+    <t>Dam örtüyü</t>
+  </si>
+  <si>
+    <t>Daxili bəzək</t>
+  </si>
+  <si>
+    <t>MEP (mex/elektrik/santexnika)</t>
+  </si>
+  <si>
+    <t>Xarici bəzək (fasad)</t>
+  </si>
+  <si>
+    <t>Təsərrüfat tikililəri</t>
+  </si>
+  <si>
+    <t>p1</t>
+  </si>
+  <si>
     <t>Paket 1 (150 ev)</t>
   </si>
   <si>
+    <t>p2</t>
+  </si>
+  <si>
     <t>Paket 2 (200 ev)</t>
   </si>
   <si>
+    <t>p3</t>
+  </si>
+  <si>
     <t>Paket 3 (205 ev)</t>
   </si>
   <si>
+    <t>p4</t>
+  </si>
+  <si>
     <t>Paket 4 (296 ev)</t>
   </si>
   <si>
-    <t>p1</t>
-  </si>
-  <si>
-    <t>2 otaqlı evlər</t>
-  </si>
-  <si>
-    <t>3 otaqlı evlər</t>
-  </si>
-  <si>
-    <t>4 otaqlı evlər</t>
-  </si>
-  <si>
-    <t>5 otaqlı evlər</t>
-  </si>
-  <si>
-    <t>p2</t>
-  </si>
-  <si>
-    <t>p3</t>
-  </si>
-  <si>
-    <t>p4</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -375,7 +381,7 @@
     <t>packagesTrendNote</t>
   </si>
   <si>
-    <t>Ümumi icra: faktiki (qırmızı) və plan (mavi nöqtəli). Mənbə: həftəlik gecikmə hesabatı (21.05.2026 və 11.06.2026 kəsimləri). Aralıq həftələr üçün yalnız gecikmə faizi mövcuddur.</t>
+    <t>Yalnız ÜMUMİ icra. Qırmızı = faktiki, mavi nöqtəli = plan. Mənbə: həftəlik hesabatlar (28.05, 04.06, 11.06). Plan 49.64% → 54.86% qalxdığı, faktiki isə 30.17% → 31.52% qaldığı üçün plandan geriləmə həftədən-həftəyə artır.</t>
   </si>
   <si>
     <t>otherAsOf</t>
@@ -912,28 +918,28 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11">
-        <v>395</v>
+        <v>415</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>172</v>
@@ -941,7 +947,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14">
         <v>31.52</v>
@@ -949,7 +955,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15">
         <v>54.86</v>
@@ -957,26 +963,26 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
         <v>25</v>
-      </c>
-      <c r="B16" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" t="s">
         <v>27</v>
-      </c>
-      <c r="B17" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
         <v>29</v>
-      </c>
-      <c r="B18" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -995,16 +1001,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1023,10 +1029,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1054,31 +1060,31 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -1086,7 +1092,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B6">
         <v>53.24</v>
@@ -1094,7 +1100,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B7">
         <v>12.31</v>
@@ -1102,31 +1108,31 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -1134,58 +1140,58 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B13" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B14" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B15" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1204,51 +1210,51 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>40</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>41</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>42</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>43</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>44</v>
-      </c>
-      <c r="G2" t="s">
-        <v>45</v>
       </c>
       <c r="H2" t="b">
         <v>0</v>
@@ -1256,25 +1262,25 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
         <v>46</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>48</v>
       </c>
-      <c r="E3" t="s">
-        <v>49</v>
-      </c>
       <c r="F3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" t="s">
         <v>44</v>
-      </c>
-      <c r="G3" t="s">
-        <v>45</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -1282,25 +1288,25 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
         <v>50</v>
       </c>
-      <c r="B4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>51</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>52</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>53</v>
-      </c>
-      <c r="G4" t="s">
-        <v>54</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -1308,25 +1314,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
         <v>55</v>
       </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" t="s">
         <v>56</v>
       </c>
-      <c r="E5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" t="s">
-        <v>57</v>
-      </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -1334,25 +1340,25 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" t="s">
         <v>58</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>59</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>60</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>61</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>62</v>
       </c>
-      <c r="F6" t="s">
-        <v>63</v>
-      </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1374,18 +1380,18 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2">
         <v>55.64</v>
@@ -1396,7 +1402,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3">
         <v>70.76</v>
@@ -1407,7 +1413,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4">
         <v>62.04</v>
@@ -1418,7 +1424,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <v>44.69</v>
@@ -1429,7 +1435,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6">
         <v>45.56</v>
@@ -1440,7 +1446,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B7">
         <v>53.24</v>
@@ -1465,21 +1471,21 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B2">
         <v>150</v>
@@ -1493,7 +1499,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B3">
         <v>200</v>
@@ -1507,7 +1513,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B4">
         <v>205</v>
@@ -1521,7 +1527,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B5">
         <v>296</v>
@@ -1541,7 +1547,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="22" customWidth="1"/>
@@ -1549,34 +1555,45 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B2">
-        <v>26.05</v>
+        <v>30.17</v>
       </c>
       <c r="C2">
-        <v>45.66</v>
+        <v>49.64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3">
+        <v>31.03</v>
+      </c>
+      <c r="C3">
+        <v>51.74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>31.52</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>54.86</v>
       </c>
     </row>
@@ -1588,7 +1605,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -1608,10 +1625,10 @@
         <v>79</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1628,10 +1645,10 @@
         <v>82</v>
       </c>
       <c r="E2">
-        <v>70.76</v>
+        <v>89.8</v>
       </c>
       <c r="F2">
-        <v>52.92</v>
+        <v>84.26</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1648,10 +1665,10 @@
         <v>83</v>
       </c>
       <c r="E3">
-        <v>62.04</v>
+        <v>21.79</v>
       </c>
       <c r="F3">
-        <v>42.49</v>
+        <v>6.69</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1668,10 +1685,10 @@
         <v>84</v>
       </c>
       <c r="E4">
-        <v>44.69</v>
+        <v>21.96</v>
       </c>
       <c r="F4">
-        <v>33.07</v>
+        <v>5.87</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1688,330 +1705,530 @@
         <v>85</v>
       </c>
       <c r="E5">
-        <v>45.56</v>
+        <v>32.95</v>
       </c>
       <c r="F5">
-        <v>35.18</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6">
+        <v>851</v>
+      </c>
+      <c r="D6" t="s">
         <v>86</v>
       </c>
-      <c r="B6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6">
-        <v>150</v>
-      </c>
-      <c r="D6" t="s">
-        <v>87</v>
-      </c>
       <c r="E6">
-        <v>77.93</v>
+        <v>6.43</v>
       </c>
       <c r="F6">
-        <v>56.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C7">
-        <v>150</v>
+        <v>851</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E7">
-        <v>76.73</v>
+        <v>59.46</v>
       </c>
       <c r="F7">
-        <v>57.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C8">
         <v>150</v>
       </c>
       <c r="D8" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="E8">
-        <v>59.19</v>
+        <v>98.55</v>
       </c>
       <c r="F8">
-        <v>45.12</v>
+        <v>95.56</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C9">
         <v>150</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E9">
-        <v>61.99</v>
+        <v>33.66</v>
       </c>
       <c r="F9">
-        <v>48.51</v>
+        <v>26.77</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B10" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C10">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E10">
-        <v>71.42</v>
+        <v>43.18</v>
       </c>
       <c r="F10">
-        <v>45.97</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C11">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D11" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E11">
-        <v>67</v>
+        <v>52.78</v>
       </c>
       <c r="F11">
-        <v>46.51</v>
+        <v>14.86</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C12">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E12">
-        <v>56.93</v>
+        <v>9.44</v>
       </c>
       <c r="F12">
-        <v>29.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C13">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D13" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E13">
-        <v>40.97</v>
+        <v>59.72</v>
       </c>
       <c r="F13">
-        <v>36.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C14">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D14" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E14">
-        <v>50.76</v>
+        <v>91.66</v>
       </c>
       <c r="F14">
-        <v>38.47</v>
+        <v>88.59</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B15" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C15">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D15" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E15">
-        <v>37.75</v>
+        <v>40.54</v>
       </c>
       <c r="F15">
-        <v>30.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16">
+        <v>200</v>
+      </c>
+      <c r="D16" t="s">
         <v>84</v>
       </c>
-      <c r="C16">
-        <v>205</v>
-      </c>
-      <c r="D16" t="s">
-        <v>89</v>
-      </c>
       <c r="E16">
-        <v>46.49</v>
+        <v>24.27</v>
       </c>
       <c r="F16">
-        <v>31.26</v>
+        <v>7.74</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C17">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D17" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E17">
-        <v>42.3</v>
+        <v>42.09</v>
       </c>
       <c r="F17">
-        <v>31.08</v>
+        <v>7.96</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C18">
-        <v>296</v>
+        <v>200</v>
       </c>
       <c r="D18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E18">
-        <v>54.98</v>
+        <v>15.5</v>
       </c>
       <c r="F18">
-        <v>25.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C19">
-        <v>296</v>
+        <v>200</v>
       </c>
       <c r="D19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E19">
-        <v>41.2</v>
+        <v>66.28</v>
       </c>
       <c r="F19">
-        <v>46.98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" t="s">
         <v>93</v>
       </c>
-      <c r="B20" t="s">
-        <v>85</v>
-      </c>
       <c r="C20">
-        <v>296</v>
+        <v>205</v>
       </c>
       <c r="D20" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="E20">
-        <v>48.88</v>
+        <v>84.77</v>
       </c>
       <c r="F20">
-        <v>34.24</v>
+        <v>74.53</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" t="s">
         <v>93</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21">
+        <v>205</v>
+      </c>
+      <c r="D21" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22">
+        <v>205</v>
+      </c>
+      <c r="D22" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22">
+        <v>8.7</v>
+      </c>
+      <c r="F22">
+        <v>4.31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>92</v>
+      </c>
+      <c r="B23" t="s">
+        <v>93</v>
+      </c>
+      <c r="C23">
+        <v>205</v>
+      </c>
+      <c r="D23" t="s">
         <v>85</v>
       </c>
-      <c r="C21">
+      <c r="E23">
+        <v>22.88</v>
+      </c>
+      <c r="F23">
+        <v>7.42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24">
+        <v>205</v>
+      </c>
+      <c r="D24" t="s">
+        <v>86</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25">
+        <v>205</v>
+      </c>
+      <c r="D25" t="s">
+        <v>87</v>
+      </c>
+      <c r="E25">
+        <v>55.93</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26">
         <v>296</v>
       </c>
-      <c r="D21" t="s">
-        <v>90</v>
-      </c>
-      <c r="E21">
-        <v>33.77</v>
-      </c>
-      <c r="F21">
-        <v>31.17</v>
+      <c r="D26" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26">
+        <v>84.21</v>
+      </c>
+      <c r="F26">
+        <v>78.36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27">
+        <v>296</v>
+      </c>
+      <c r="D27" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27">
+        <v>12.97</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28">
+        <v>296</v>
+      </c>
+      <c r="D28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28">
+        <v>11.69</v>
+      </c>
+      <c r="F28">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" t="s">
+        <v>95</v>
+      </c>
+      <c r="C29">
+        <v>296</v>
+      </c>
+      <c r="D29" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29">
+        <v>14.05</v>
+      </c>
+      <c r="F29">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30">
+        <v>296</v>
+      </c>
+      <c r="D30" t="s">
+        <v>86</v>
+      </c>
+      <c r="E30">
+        <v>0.78</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" t="s">
+        <v>95</v>
+      </c>
+      <c r="C31">
+        <v>296</v>
+      </c>
+      <c r="D31" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31">
+        <v>55.93</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2030,16 +2247,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2058,18 +2275,18 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B2">
         <v>44.64</v>
@@ -2080,7 +2297,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B3">
         <v>41.2</v>
@@ -2091,7 +2308,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B4">
         <v>52.54</v>
@@ -2102,7 +2319,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B5">
         <v>69.53</v>
@@ -2127,33 +2344,33 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B2">
         <v>54.86</v>
@@ -2162,7 +2379,7 @@
         <v>31.52</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E2">
         <v>26.05</v>
@@ -2179,7 +2396,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B3">
         <v>55.64</v>
@@ -2188,7 +2405,7 @@
         <v>40.9</v>
       </c>
       <c r="D3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E3">
         <v>35.24</v>
@@ -2205,7 +2422,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B4">
         <v>70.76</v>
@@ -2214,7 +2431,7 @@
         <v>52.92</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E4">
         <v>48.13</v>
@@ -2231,7 +2448,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B5">
         <v>62.04</v>
@@ -2240,7 +2457,7 @@
         <v>42.49</v>
       </c>
       <c r="D5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E5">
         <v>38.28</v>
@@ -2257,7 +2474,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B6">
         <v>44.69</v>
@@ -2266,7 +2483,7 @@
         <v>33.07</v>
       </c>
       <c r="D6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E6">
         <v>25.81</v>
@@ -2283,7 +2500,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="B7">
         <v>45.56</v>
@@ -2292,7 +2509,7 @@
         <v>35.18</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E7">
         <v>28.76</v>
@@ -2309,7 +2526,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B8">
         <v>53.24</v>
@@ -2318,7 +2535,7 @@
         <v>12.31</v>
       </c>
       <c r="D8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E8">
         <v>7.25</v>

</xml_diff>

<commit_message>
Detailed Görülən işlər + Infrastruktur, tempo help, weekly-change chart
Görülən işlər: now drills to each house type (2/3/4/5 otaqlı) per packet, with
the 6 work stages (Qaba işlər, Dam örtüyü, Daxili bəzək, MEP, Xarici bəzək,
Təsərrüfat) showing BOTH plan and fakt (grouped bars). 21 tabs (Cəmi, per-packet
average, and 16 room-level). Data = real Primavera WBS Performance%/Schedule%.

İnfrastruktur İcrası: phase tabs (Mərhələ 1-4 + overview); each phase shows all
8 utilities (su kanalizasiya, su şəbəkəsi, qaz, 35/0.4 kV kabel, rabitə, PTM/KTM,
yollar) with plan and fakt.

Həftəlik tempo: added a '?' with the Tələb/Faktiki formula explanation.

Həftəlik sürət: added a weekly delay-change chart (04.06→11.06) per object —
gecikmə artması (red) / azalması (green), from the Excel həftəlik dəyişiklik
column (e.g. Ümumi +2.63%, Paket 1 +3.17%).

Schema: round-trips infrastructure.lots (new InfraItems sheet) in both the Node
build and the app exporter. Nothing else changed. All tests pass.
</commit_message>
<xml_diff>
--- a/cities/qervend/source.xlsx
+++ b/cities/qervend/source.xlsx
@@ -12,17 +12,18 @@
     <sheet sheetId="6" name="WorkItems" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Other" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Infrastructure" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Velocity" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="WorkforceDaily" state="visible" r:id="rId13"/>
-    <sheet sheetId="11" name="WorkforceMachinery" state="visible" r:id="rId14"/>
-    <sheet sheetId="12" name="Notes" state="visible" r:id="rId15"/>
+    <sheet sheetId="9" name="InfraItems" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Velocity" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="WorkforceDaily" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="WorkforceMachinery" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="Notes" state="visible" r:id="rId16"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="193">
   <si>
     <t>Sahə</t>
   </si>
@@ -279,90 +280,237 @@
     <t>Daxili bəzək</t>
   </si>
   <si>
-    <t>MEP (mex/elektrik/santexnika)</t>
-  </si>
-  <si>
-    <t>Xarici bəzək (fasad)</t>
-  </si>
-  <si>
-    <t>Təsərrüfat tikililəri</t>
+    <t>MEP</t>
+  </si>
+  <si>
+    <t>Xarici bəzək</t>
+  </si>
+  <si>
+    <t>Təsərrüfat</t>
   </si>
   <si>
     <t>p1</t>
   </si>
   <si>
+    <t>Paket 1 (150 ev) — orta</t>
+  </si>
+  <si>
+    <t>p1r1</t>
+  </si>
+  <si>
+    <t>Paket 1 — 2 otaqlı</t>
+  </si>
+  <si>
+    <t>p1r2</t>
+  </si>
+  <si>
+    <t>Paket 1 — 3 otaqlı</t>
+  </si>
+  <si>
+    <t>p1r3</t>
+  </si>
+  <si>
+    <t>Paket 1 — 4 otaqlı</t>
+  </si>
+  <si>
+    <t>p1r4</t>
+  </si>
+  <si>
+    <t>Paket 1 — 5 otaqlı</t>
+  </si>
+  <si>
+    <t>p2</t>
+  </si>
+  <si>
+    <t>Paket 2 (200 ev) — orta</t>
+  </si>
+  <si>
+    <t>p2r1</t>
+  </si>
+  <si>
+    <t>Paket 2 — 2 otaqlı</t>
+  </si>
+  <si>
+    <t>p2r2</t>
+  </si>
+  <si>
+    <t>Paket 2 — 3 otaqlı</t>
+  </si>
+  <si>
+    <t>p2r3</t>
+  </si>
+  <si>
+    <t>Paket 2 — 4 otaqlı</t>
+  </si>
+  <si>
+    <t>p2r4</t>
+  </si>
+  <si>
+    <t>Paket 2 — 5 otaqlı</t>
+  </si>
+  <si>
+    <t>p3</t>
+  </si>
+  <si>
+    <t>Paket 3 (205 ev) — orta</t>
+  </si>
+  <si>
+    <t>p3r1</t>
+  </si>
+  <si>
+    <t>Paket 3 — 2 otaqlı</t>
+  </si>
+  <si>
+    <t>p3r2</t>
+  </si>
+  <si>
+    <t>Paket 3 — 3 otaqlı</t>
+  </si>
+  <si>
+    <t>p3r3</t>
+  </si>
+  <si>
+    <t>Paket 3 — 4 otaqlı</t>
+  </si>
+  <si>
+    <t>p3r4</t>
+  </si>
+  <si>
+    <t>Paket 3 — 5 otaqlı</t>
+  </si>
+  <si>
+    <t>p4</t>
+  </si>
+  <si>
+    <t>Paket 4 (296 ev) — orta</t>
+  </si>
+  <si>
+    <t>p4r1</t>
+  </si>
+  <si>
+    <t>Paket 4 — 2 otaqlı</t>
+  </si>
+  <si>
+    <t>p4r2</t>
+  </si>
+  <si>
+    <t>Paket 4 — 3 otaqlı</t>
+  </si>
+  <si>
+    <t>p4r3</t>
+  </si>
+  <si>
+    <t>Paket 4 — 4 otaqlı</t>
+  </si>
+  <si>
+    <t>p4r4</t>
+  </si>
+  <si>
+    <t>Paket 4 — 5 otaqlı</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Mərhələ 1</t>
+  </si>
+  <si>
+    <t>Mərhələ 2</t>
+  </si>
+  <si>
+    <t>Mərhələ 3</t>
+  </si>
+  <si>
+    <t>Mərhələ 4</t>
+  </si>
+  <si>
+    <t>Mərhələ üzrə</t>
+  </si>
+  <si>
+    <t>m1</t>
+  </si>
+  <si>
+    <t>Xarici su kanalizasiyası</t>
+  </si>
+  <si>
+    <t>Xarici su şəbəkəsi</t>
+  </si>
+  <si>
+    <t>Qaz təchizatı</t>
+  </si>
+  <si>
+    <t>35 kV kabel xətti</t>
+  </si>
+  <si>
+    <t>0.4 kV kabel xətti</t>
+  </si>
+  <si>
+    <t>Rabitə şəbəkəsi</t>
+  </si>
+  <si>
+    <t>PTM və KTM</t>
+  </si>
+  <si>
+    <t>Yollar və səkilər</t>
+  </si>
+  <si>
+    <t>m2</t>
+  </si>
+  <si>
+    <t>m3</t>
+  </si>
+  <si>
+    <t>m4</t>
+  </si>
+  <si>
+    <t>obyekt</t>
+  </si>
+  <si>
+    <t>finish</t>
+  </si>
+  <si>
+    <t>priorFakt</t>
+  </si>
+  <si>
+    <t>dev1</t>
+  </si>
+  <si>
+    <t>dev2</t>
+  </si>
+  <si>
+    <t>dev3</t>
+  </si>
+  <si>
+    <t>Ümumi</t>
+  </si>
+  <si>
+    <t>2026-11-30</t>
+  </si>
+  <si>
+    <t>FYE (851 ev)</t>
+  </si>
+  <si>
     <t>Paket 1 (150 ev)</t>
   </si>
   <si>
-    <t>p2</t>
+    <t>2026-09-30</t>
   </si>
   <si>
     <t>Paket 2 (200 ev)</t>
   </si>
   <si>
-    <t>p3</t>
+    <t>2026-10-31</t>
   </si>
   <si>
     <t>Paket 3 (205 ev)</t>
   </si>
   <si>
-    <t>p4</t>
+    <t>2026-11-15</t>
   </si>
   <si>
     <t>Paket 4 (296 ev)</t>
   </si>
   <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>Mərhələ 1</t>
-  </si>
-  <si>
-    <t>Mərhələ 2</t>
-  </si>
-  <si>
-    <t>Mərhələ 3</t>
-  </si>
-  <si>
-    <t>Mərhələ 4</t>
-  </si>
-  <si>
-    <t>obyekt</t>
-  </si>
-  <si>
-    <t>finish</t>
-  </si>
-  <si>
-    <t>priorFakt</t>
-  </si>
-  <si>
-    <t>dev1</t>
-  </si>
-  <si>
-    <t>dev2</t>
-  </si>
-  <si>
-    <t>dev3</t>
-  </si>
-  <si>
-    <t>Ümumi</t>
-  </si>
-  <si>
-    <t>2026-11-30</t>
-  </si>
-  <si>
-    <t>FYE (851 ev)</t>
-  </si>
-  <si>
-    <t>2026-09-30</t>
-  </si>
-  <si>
-    <t>2026-10-31</t>
-  </si>
-  <si>
-    <t>2026-11-15</t>
-  </si>
-  <si>
     <t>Sahədaxili komm.</t>
   </si>
   <si>
@@ -402,7 +550,7 @@
     <t>infraWeeklyNote</t>
   </si>
   <si>
-    <t>Sahədaxili kommunikasiya üzrə ümumi icra 11.06 tarixinə 12.31% təşkil edir və plandan 40.93% geri qalır. Hər mərhələ daxilində yollar, kanalizasiya, su, qaz, elektrik (35/0.4 kV) və rabitə şəbəkələri ayrıca izlənilir; yalnız yollar və kanalizasiya üzrə məhdud irəliləyiş var, qalan şəbəkələr faktiki olaraq başlanmamışdır.</t>
+    <t>Sahədaxili kommunikasiya üzrə ümumi icra 12.31%, plandan 40.93% geri. Hər mərhələ daxilində yollar, kanalizasiya, su, qaz, elektrik və rabitə ayrıca izlənilir.</t>
   </si>
   <si>
     <t>velCutoff</t>
@@ -993,6 +1141,228 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2">
+        <v>54.86</v>
+      </c>
+      <c r="C2">
+        <v>31.52</v>
+      </c>
+      <c r="D2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E2">
+        <v>26.05</v>
+      </c>
+      <c r="F2">
+        <v>-19.47</v>
+      </c>
+      <c r="G2">
+        <v>-20.71</v>
+      </c>
+      <c r="H2">
+        <v>-23.34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3">
+        <v>55.64</v>
+      </c>
+      <c r="C3">
+        <v>40.9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3">
+        <v>35.24</v>
+      </c>
+      <c r="F3">
+        <v>-10.65</v>
+      </c>
+      <c r="G3">
+        <v>-12.4</v>
+      </c>
+      <c r="H3">
+        <v>-14.74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4">
+        <v>70.76</v>
+      </c>
+      <c r="C4">
+        <v>52.92</v>
+      </c>
+      <c r="D4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4">
+        <v>48.13</v>
+      </c>
+      <c r="F4">
+        <v>-12.25</v>
+      </c>
+      <c r="G4">
+        <v>-14.67</v>
+      </c>
+      <c r="H4">
+        <v>-17.84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5">
+        <v>62.04</v>
+      </c>
+      <c r="C5">
+        <v>42.49</v>
+      </c>
+      <c r="D5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5">
+        <v>38.28</v>
+      </c>
+      <c r="F5">
+        <v>-15.03</v>
+      </c>
+      <c r="G5">
+        <v>-17.2</v>
+      </c>
+      <c r="H5">
+        <v>-19.55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6">
+        <v>44.69</v>
+      </c>
+      <c r="C6">
+        <v>33.07</v>
+      </c>
+      <c r="D6" t="s">
+        <v>160</v>
+      </c>
+      <c r="E6">
+        <v>25.81</v>
+      </c>
+      <c r="F6">
+        <v>-7.76</v>
+      </c>
+      <c r="G6">
+        <v>-9.25</v>
+      </c>
+      <c r="H6">
+        <v>-11.89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B7">
+        <v>45.56</v>
+      </c>
+      <c r="C7">
+        <v>35.18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7">
+        <v>28.76</v>
+      </c>
+      <c r="F7">
+        <v>-7.78</v>
+      </c>
+      <c r="G7">
+        <v>-8.77</v>
+      </c>
+      <c r="H7">
+        <v>-10.38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B8">
+        <v>53.24</v>
+      </c>
+      <c r="C8">
+        <v>12.31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>153</v>
+      </c>
+      <c r="E8">
+        <v>7.25</v>
+      </c>
+      <c r="F8">
+        <v>-37.51</v>
+      </c>
+      <c r="G8">
+        <v>-37.71</v>
+      </c>
+      <c r="H8">
+        <v>-40.93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1004,13 +1374,13 @@
         <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>115</v>
+        <v>164</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>116</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -1019,7 +1389,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1032,7 +1402,7 @@
         <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>117</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -1041,7 +1411,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1060,15 +1430,15 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>167</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>120</v>
+        <v>169</v>
       </c>
       <c r="B3" t="s">
         <v>27</v>
@@ -1076,7 +1446,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>121</v>
+        <v>170</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
@@ -1084,7 +1454,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -1092,7 +1462,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>123</v>
+        <v>172</v>
       </c>
       <c r="B6">
         <v>53.24</v>
@@ -1100,7 +1470,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>124</v>
+        <v>173</v>
       </c>
       <c r="B7">
         <v>12.31</v>
@@ -1108,31 +1478,31 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>125</v>
+        <v>174</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="B9" t="s">
-        <v>128</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>129</v>
+        <v>178</v>
       </c>
       <c r="B10" t="s">
-        <v>130</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>180</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -1140,39 +1510,39 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="B12" t="s">
-        <v>133</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>134</v>
+        <v>183</v>
       </c>
       <c r="B13" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="B14" t="s">
-        <v>137</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="B15" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>140</v>
+        <v>189</v>
       </c>
       <c r="B16" t="s">
         <v>27</v>
@@ -1180,15 +1550,15 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>141</v>
+        <v>190</v>
       </c>
       <c r="B17" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>143</v>
+        <v>192</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
@@ -1605,7 +1975,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -1878,17 +2248,14 @@
       <c r="B14" t="s">
         <v>91</v>
       </c>
-      <c r="C14">
-        <v>200</v>
-      </c>
       <c r="D14" t="s">
         <v>82</v>
       </c>
       <c r="E14">
-        <v>91.66</v>
+        <v>100</v>
       </c>
       <c r="F14">
-        <v>88.59</v>
+        <v>94.7</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1898,17 +2265,14 @@
       <c r="B15" t="s">
         <v>91</v>
       </c>
-      <c r="C15">
-        <v>200</v>
-      </c>
       <c r="D15" t="s">
         <v>83</v>
       </c>
       <c r="E15">
-        <v>40.54</v>
+        <v>83.87</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>8.29</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1918,17 +2282,14 @@
       <c r="B16" t="s">
         <v>91</v>
       </c>
-      <c r="C16">
-        <v>200</v>
-      </c>
       <c r="D16" t="s">
         <v>84</v>
       </c>
       <c r="E16">
-        <v>24.27</v>
+        <v>67.94</v>
       </c>
       <c r="F16">
-        <v>7.74</v>
+        <v>6.74</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1938,17 +2299,14 @@
       <c r="B17" t="s">
         <v>91</v>
       </c>
-      <c r="C17">
-        <v>200</v>
-      </c>
       <c r="D17" t="s">
         <v>85</v>
       </c>
       <c r="E17">
-        <v>42.09</v>
+        <v>50.57</v>
       </c>
       <c r="F17">
-        <v>7.96</v>
+        <v>5.61</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1958,14 +2316,11 @@
       <c r="B18" t="s">
         <v>91</v>
       </c>
-      <c r="C18">
-        <v>200</v>
-      </c>
       <c r="D18" t="s">
         <v>86</v>
       </c>
       <c r="E18">
-        <v>15.5</v>
+        <v>34.23</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1978,14 +2333,11 @@
       <c r="B19" t="s">
         <v>91</v>
       </c>
-      <c r="C19">
-        <v>200</v>
-      </c>
       <c r="D19" t="s">
         <v>87</v>
       </c>
       <c r="E19">
-        <v>66.28</v>
+        <v>9.01</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1998,17 +2350,14 @@
       <c r="B20" t="s">
         <v>93</v>
       </c>
-      <c r="C20">
-        <v>205</v>
-      </c>
       <c r="D20" t="s">
         <v>82</v>
       </c>
       <c r="E20">
-        <v>84.77</v>
+        <v>99.12</v>
       </c>
       <c r="F20">
-        <v>74.53</v>
+        <v>97.33</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -2018,17 +2367,14 @@
       <c r="B21" t="s">
         <v>93</v>
       </c>
-      <c r="C21">
-        <v>205</v>
-      </c>
       <c r="D21" t="s">
         <v>83</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>30.55</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>11.56</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -2038,17 +2384,14 @@
       <c r="B22" t="s">
         <v>93</v>
       </c>
-      <c r="C22">
-        <v>205</v>
-      </c>
       <c r="D22" t="s">
         <v>84</v>
       </c>
       <c r="E22">
-        <v>8.7</v>
+        <v>60.88</v>
       </c>
       <c r="F22">
-        <v>4.31</v>
+        <v>10.35</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2058,17 +2401,14 @@
       <c r="B23" t="s">
         <v>93</v>
       </c>
-      <c r="C23">
-        <v>205</v>
-      </c>
       <c r="D23" t="s">
         <v>85</v>
       </c>
       <c r="E23">
-        <v>22.88</v>
+        <v>68.06</v>
       </c>
       <c r="F23">
-        <v>7.42</v>
+        <v>19.04</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2078,14 +2418,11 @@
       <c r="B24" t="s">
         <v>93</v>
       </c>
-      <c r="C24">
-        <v>205</v>
-      </c>
       <c r="D24" t="s">
         <v>86</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>1.11</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -2098,14 +2435,11 @@
       <c r="B25" t="s">
         <v>93</v>
       </c>
-      <c r="C25">
-        <v>205</v>
-      </c>
       <c r="D25" t="s">
         <v>87</v>
       </c>
       <c r="E25">
-        <v>55.93</v>
+        <v>76.62</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -2118,17 +2452,14 @@
       <c r="B26" t="s">
         <v>95</v>
       </c>
-      <c r="C26">
-        <v>296</v>
-      </c>
       <c r="D26" t="s">
         <v>82</v>
       </c>
       <c r="E26">
-        <v>84.21</v>
+        <v>96.65</v>
       </c>
       <c r="F26">
-        <v>78.36</v>
+        <v>94.47</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2138,17 +2469,14 @@
       <c r="B27" t="s">
         <v>95</v>
       </c>
-      <c r="C27">
-        <v>296</v>
-      </c>
       <c r="D27" t="s">
         <v>83</v>
       </c>
       <c r="E27">
-        <v>12.97</v>
+        <v>0</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>9.51</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2158,17 +2486,14 @@
       <c r="B28" t="s">
         <v>95</v>
       </c>
-      <c r="C28">
-        <v>296</v>
-      </c>
       <c r="D28" t="s">
         <v>84</v>
       </c>
       <c r="E28">
-        <v>11.69</v>
+        <v>20.41</v>
       </c>
       <c r="F28">
-        <v>3.33</v>
+        <v>8.41</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2178,17 +2503,14 @@
       <c r="B29" t="s">
         <v>95</v>
       </c>
-      <c r="C29">
-        <v>296</v>
-      </c>
       <c r="D29" t="s">
         <v>85</v>
       </c>
       <c r="E29">
-        <v>14.05</v>
+        <v>43.91</v>
       </c>
       <c r="F29">
-        <v>0.61</v>
+        <v>13.97</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2198,14 +2520,11 @@
       <c r="B30" t="s">
         <v>95</v>
       </c>
-      <c r="C30">
-        <v>296</v>
-      </c>
       <c r="D30" t="s">
         <v>86</v>
       </c>
       <c r="E30">
-        <v>0.78</v>
+        <v>0</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -2218,16 +2537,1699 @@
       <c r="B31" t="s">
         <v>95</v>
       </c>
-      <c r="C31">
-        <v>296</v>
-      </c>
       <c r="D31" t="s">
         <v>87</v>
       </c>
       <c r="E31">
+        <v>76.62</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B32" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E32">
+        <v>98.43</v>
+      </c>
+      <c r="F32">
+        <v>95.74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" t="s">
+        <v>83</v>
+      </c>
+      <c r="E33">
+        <v>20.24</v>
+      </c>
+      <c r="F33">
+        <v>77.71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>96</v>
+      </c>
+      <c r="B34" t="s">
+        <v>97</v>
+      </c>
+      <c r="D34" t="s">
+        <v>84</v>
+      </c>
+      <c r="E34">
+        <v>23.5</v>
+      </c>
+      <c r="F34">
+        <v>6.88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="D35" t="s">
+        <v>85</v>
+      </c>
+      <c r="E35">
+        <v>48.58</v>
+      </c>
+      <c r="F35">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" t="s">
+        <v>97</v>
+      </c>
+      <c r="D36" t="s">
+        <v>86</v>
+      </c>
+      <c r="E36">
+        <v>2.44</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>96</v>
+      </c>
+      <c r="B37" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" t="s">
+        <v>87</v>
+      </c>
+      <c r="E37">
+        <v>76.62</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38">
+        <v>200</v>
+      </c>
+      <c r="D38" t="s">
+        <v>82</v>
+      </c>
+      <c r="E38">
+        <v>91.66</v>
+      </c>
+      <c r="F38">
+        <v>88.59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39">
+        <v>200</v>
+      </c>
+      <c r="D39" t="s">
+        <v>83</v>
+      </c>
+      <c r="E39">
+        <v>40.54</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>98</v>
+      </c>
+      <c r="B40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40">
+        <v>200</v>
+      </c>
+      <c r="D40" t="s">
+        <v>84</v>
+      </c>
+      <c r="E40">
+        <v>24.27</v>
+      </c>
+      <c r="F40">
+        <v>7.74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" t="s">
+        <v>99</v>
+      </c>
+      <c r="C41">
+        <v>200</v>
+      </c>
+      <c r="D41" t="s">
+        <v>85</v>
+      </c>
+      <c r="E41">
+        <v>42.09</v>
+      </c>
+      <c r="F41">
+        <v>7.96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>98</v>
+      </c>
+      <c r="B42" t="s">
+        <v>99</v>
+      </c>
+      <c r="C42">
+        <v>200</v>
+      </c>
+      <c r="D42" t="s">
+        <v>86</v>
+      </c>
+      <c r="E42">
+        <v>15.5</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>98</v>
+      </c>
+      <c r="B43" t="s">
+        <v>99</v>
+      </c>
+      <c r="C43">
+        <v>200</v>
+      </c>
+      <c r="D43" t="s">
+        <v>87</v>
+      </c>
+      <c r="E43">
+        <v>66.28</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>100</v>
+      </c>
+      <c r="B44" t="s">
+        <v>101</v>
+      </c>
+      <c r="D44" t="s">
+        <v>82</v>
+      </c>
+      <c r="E44">
+        <v>100</v>
+      </c>
+      <c r="F44">
+        <v>94.09</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>100</v>
+      </c>
+      <c r="B45" t="s">
+        <v>101</v>
+      </c>
+      <c r="D45" t="s">
+        <v>83</v>
+      </c>
+      <c r="E45">
+        <v>100</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>100</v>
+      </c>
+      <c r="B46" t="s">
+        <v>101</v>
+      </c>
+      <c r="D46" t="s">
+        <v>84</v>
+      </c>
+      <c r="E46">
+        <v>36.63</v>
+      </c>
+      <c r="F46">
+        <v>7.92</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>100</v>
+      </c>
+      <c r="B47" t="s">
+        <v>101</v>
+      </c>
+      <c r="D47" t="s">
+        <v>85</v>
+      </c>
+      <c r="E47">
+        <v>51.75</v>
+      </c>
+      <c r="F47">
+        <v>3.34</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>100</v>
+      </c>
+      <c r="B48" t="s">
+        <v>101</v>
+      </c>
+      <c r="D48" t="s">
+        <v>86</v>
+      </c>
+      <c r="E48">
+        <v>14.8</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>100</v>
+      </c>
+      <c r="B49" t="s">
+        <v>101</v>
+      </c>
+      <c r="D49" t="s">
+        <v>87</v>
+      </c>
+      <c r="E49">
+        <v>76.62</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" t="s">
+        <v>103</v>
+      </c>
+      <c r="D50" t="s">
+        <v>82</v>
+      </c>
+      <c r="E50">
+        <v>97.81</v>
+      </c>
+      <c r="F50">
+        <v>92.72</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>102</v>
+      </c>
+      <c r="B51" t="s">
+        <v>103</v>
+      </c>
+      <c r="D51" t="s">
+        <v>83</v>
+      </c>
+      <c r="E51">
+        <v>62.15</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" t="s">
+        <v>103</v>
+      </c>
+      <c r="D52" t="s">
+        <v>84</v>
+      </c>
+      <c r="E52">
+        <v>34.16</v>
+      </c>
+      <c r="F52">
+        <v>11.13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>102</v>
+      </c>
+      <c r="B53" t="s">
+        <v>103</v>
+      </c>
+      <c r="D53" t="s">
+        <v>85</v>
+      </c>
+      <c r="E53">
+        <v>46.28</v>
+      </c>
+      <c r="F53">
+        <v>18.13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" t="s">
+        <v>103</v>
+      </c>
+      <c r="D54" t="s">
+        <v>86</v>
+      </c>
+      <c r="E54">
+        <v>35.63</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>102</v>
+      </c>
+      <c r="B55" t="s">
+        <v>103</v>
+      </c>
+      <c r="D55" t="s">
+        <v>87</v>
+      </c>
+      <c r="E55">
+        <v>76.62</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>104</v>
+      </c>
+      <c r="B56" t="s">
+        <v>105</v>
+      </c>
+      <c r="D56" t="s">
+        <v>82</v>
+      </c>
+      <c r="E56">
+        <v>89.33</v>
+      </c>
+      <c r="F56">
+        <v>90.36</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>104</v>
+      </c>
+      <c r="B57" t="s">
+        <v>105</v>
+      </c>
+      <c r="D57" t="s">
+        <v>83</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>104</v>
+      </c>
+      <c r="B58" t="s">
+        <v>105</v>
+      </c>
+      <c r="D58" t="s">
+        <v>84</v>
+      </c>
+      <c r="E58">
+        <v>26.29</v>
+      </c>
+      <c r="F58">
+        <v>9.72</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>104</v>
+      </c>
+      <c r="B59" t="s">
+        <v>105</v>
+      </c>
+      <c r="D59" t="s">
+        <v>85</v>
+      </c>
+      <c r="E59">
+        <v>70.33</v>
+      </c>
+      <c r="F59">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>104</v>
+      </c>
+      <c r="B60" t="s">
+        <v>105</v>
+      </c>
+      <c r="D60" t="s">
+        <v>86</v>
+      </c>
+      <c r="E60">
+        <v>11.57</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>104</v>
+      </c>
+      <c r="B61" t="s">
+        <v>105</v>
+      </c>
+      <c r="D61" t="s">
+        <v>87</v>
+      </c>
+      <c r="E61">
         <v>55.93</v>
       </c>
-      <c r="F31">
+      <c r="F61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>106</v>
+      </c>
+      <c r="B62" t="s">
+        <v>107</v>
+      </c>
+      <c r="D62" t="s">
+        <v>82</v>
+      </c>
+      <c r="E62">
+        <v>79.5</v>
+      </c>
+      <c r="F62">
+        <v>77.2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>106</v>
+      </c>
+      <c r="B63" t="s">
+        <v>107</v>
+      </c>
+      <c r="D63" t="s">
+        <v>83</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>106</v>
+      </c>
+      <c r="B64" t="s">
+        <v>107</v>
+      </c>
+      <c r="D64" t="s">
+        <v>84</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>2.19</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>106</v>
+      </c>
+      <c r="B65" t="s">
+        <v>107</v>
+      </c>
+      <c r="D65" t="s">
+        <v>85</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>6.61</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>106</v>
+      </c>
+      <c r="B66" t="s">
+        <v>107</v>
+      </c>
+      <c r="D66" t="s">
+        <v>86</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>106</v>
+      </c>
+      <c r="B67" t="s">
+        <v>107</v>
+      </c>
+      <c r="D67" t="s">
+        <v>87</v>
+      </c>
+      <c r="E67">
+        <v>55.93</v>
+      </c>
+      <c r="F67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>108</v>
+      </c>
+      <c r="B68" t="s">
+        <v>109</v>
+      </c>
+      <c r="C68">
+        <v>205</v>
+      </c>
+      <c r="D68" t="s">
+        <v>82</v>
+      </c>
+      <c r="E68">
+        <v>84.77</v>
+      </c>
+      <c r="F68">
+        <v>74.53</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>108</v>
+      </c>
+      <c r="B69" t="s">
+        <v>109</v>
+      </c>
+      <c r="C69">
+        <v>205</v>
+      </c>
+      <c r="D69" t="s">
+        <v>83</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>108</v>
+      </c>
+      <c r="B70" t="s">
+        <v>109</v>
+      </c>
+      <c r="C70">
+        <v>205</v>
+      </c>
+      <c r="D70" t="s">
+        <v>84</v>
+      </c>
+      <c r="E70">
+        <v>8.7</v>
+      </c>
+      <c r="F70">
+        <v>4.31</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>108</v>
+      </c>
+      <c r="B71" t="s">
+        <v>109</v>
+      </c>
+      <c r="C71">
+        <v>205</v>
+      </c>
+      <c r="D71" t="s">
+        <v>85</v>
+      </c>
+      <c r="E71">
+        <v>22.88</v>
+      </c>
+      <c r="F71">
+        <v>7.42</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>108</v>
+      </c>
+      <c r="B72" t="s">
+        <v>109</v>
+      </c>
+      <c r="C72">
+        <v>205</v>
+      </c>
+      <c r="D72" t="s">
+        <v>86</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>108</v>
+      </c>
+      <c r="B73" t="s">
+        <v>109</v>
+      </c>
+      <c r="C73">
+        <v>205</v>
+      </c>
+      <c r="D73" t="s">
+        <v>87</v>
+      </c>
+      <c r="E73">
+        <v>55.93</v>
+      </c>
+      <c r="F73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>110</v>
+      </c>
+      <c r="B74" t="s">
+        <v>111</v>
+      </c>
+      <c r="D74" t="s">
+        <v>82</v>
+      </c>
+      <c r="E74">
+        <v>89.54</v>
+      </c>
+      <c r="F74">
+        <v>78.95</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>110</v>
+      </c>
+      <c r="B75" t="s">
+        <v>111</v>
+      </c>
+      <c r="D75" t="s">
+        <v>83</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>110</v>
+      </c>
+      <c r="B76" t="s">
+        <v>111</v>
+      </c>
+      <c r="D76" t="s">
+        <v>84</v>
+      </c>
+      <c r="E76">
+        <v>8.68</v>
+      </c>
+      <c r="F76">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>110</v>
+      </c>
+      <c r="B77" t="s">
+        <v>111</v>
+      </c>
+      <c r="D77" t="s">
+        <v>85</v>
+      </c>
+      <c r="E77">
+        <v>23.96</v>
+      </c>
+      <c r="F77">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" t="s">
+        <v>111</v>
+      </c>
+      <c r="D78" t="s">
+        <v>86</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>110</v>
+      </c>
+      <c r="B79" t="s">
+        <v>111</v>
+      </c>
+      <c r="D79" t="s">
+        <v>87</v>
+      </c>
+      <c r="E79">
+        <v>55.93</v>
+      </c>
+      <c r="F79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>112</v>
+      </c>
+      <c r="B80" t="s">
+        <v>113</v>
+      </c>
+      <c r="D80" t="s">
+        <v>82</v>
+      </c>
+      <c r="E80">
+        <v>80.91</v>
+      </c>
+      <c r="F80">
+        <v>78.78</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>112</v>
+      </c>
+      <c r="B81" t="s">
+        <v>113</v>
+      </c>
+      <c r="D81" t="s">
+        <v>83</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>112</v>
+      </c>
+      <c r="B82" t="s">
+        <v>113</v>
+      </c>
+      <c r="D82" t="s">
+        <v>84</v>
+      </c>
+      <c r="E82">
+        <v>8.78</v>
+      </c>
+      <c r="F82">
+        <v>7.97</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83" t="s">
+        <v>113</v>
+      </c>
+      <c r="D83" t="s">
+        <v>85</v>
+      </c>
+      <c r="E83">
+        <v>27.33</v>
+      </c>
+      <c r="F83">
+        <v>14.65</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84" t="s">
+        <v>113</v>
+      </c>
+      <c r="D84" t="s">
+        <v>86</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>112</v>
+      </c>
+      <c r="B85" t="s">
+        <v>113</v>
+      </c>
+      <c r="D85" t="s">
+        <v>87</v>
+      </c>
+      <c r="E85">
+        <v>55.93</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86" t="s">
+        <v>115</v>
+      </c>
+      <c r="D86" t="s">
+        <v>82</v>
+      </c>
+      <c r="E86">
+        <v>90.05</v>
+      </c>
+      <c r="F86">
+        <v>73.01</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>114</v>
+      </c>
+      <c r="B87" t="s">
+        <v>115</v>
+      </c>
+      <c r="D87" t="s">
+        <v>83</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>114</v>
+      </c>
+      <c r="B88" t="s">
+        <v>115</v>
+      </c>
+      <c r="D88" t="s">
+        <v>84</v>
+      </c>
+      <c r="E88">
+        <v>9.02</v>
+      </c>
+      <c r="F88">
+        <v>4.44</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>114</v>
+      </c>
+      <c r="B89" t="s">
+        <v>115</v>
+      </c>
+      <c r="D89" t="s">
+        <v>85</v>
+      </c>
+      <c r="E89">
+        <v>26.55</v>
+      </c>
+      <c r="F89">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>114</v>
+      </c>
+      <c r="B90" t="s">
+        <v>115</v>
+      </c>
+      <c r="D90" t="s">
+        <v>86</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+      <c r="F90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>114</v>
+      </c>
+      <c r="B91" t="s">
+        <v>115</v>
+      </c>
+      <c r="D91" t="s">
+        <v>87</v>
+      </c>
+      <c r="E91">
+        <v>55.93</v>
+      </c>
+      <c r="F91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>116</v>
+      </c>
+      <c r="B92" t="s">
+        <v>117</v>
+      </c>
+      <c r="D92" t="s">
+        <v>82</v>
+      </c>
+      <c r="E92">
+        <v>78.56</v>
+      </c>
+      <c r="F92">
+        <v>67.4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>116</v>
+      </c>
+      <c r="B93" t="s">
+        <v>117</v>
+      </c>
+      <c r="D93" t="s">
+        <v>83</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+      <c r="F93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>116</v>
+      </c>
+      <c r="B94" t="s">
+        <v>117</v>
+      </c>
+      <c r="D94" t="s">
+        <v>84</v>
+      </c>
+      <c r="E94">
+        <v>8.3</v>
+      </c>
+      <c r="F94">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>116</v>
+      </c>
+      <c r="B95" t="s">
+        <v>117</v>
+      </c>
+      <c r="D95" t="s">
+        <v>85</v>
+      </c>
+      <c r="E95">
+        <v>13.66</v>
+      </c>
+      <c r="F95">
+        <v>8.98</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>116</v>
+      </c>
+      <c r="B96" t="s">
+        <v>117</v>
+      </c>
+      <c r="D96" t="s">
+        <v>86</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>116</v>
+      </c>
+      <c r="B97" t="s">
+        <v>117</v>
+      </c>
+      <c r="D97" t="s">
+        <v>87</v>
+      </c>
+      <c r="E97">
+        <v>55.93</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>118</v>
+      </c>
+      <c r="B98" t="s">
+        <v>119</v>
+      </c>
+      <c r="C98">
+        <v>296</v>
+      </c>
+      <c r="D98" t="s">
+        <v>82</v>
+      </c>
+      <c r="E98">
+        <v>84.21</v>
+      </c>
+      <c r="F98">
+        <v>78.36</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>118</v>
+      </c>
+      <c r="B99" t="s">
+        <v>119</v>
+      </c>
+      <c r="C99">
+        <v>296</v>
+      </c>
+      <c r="D99" t="s">
+        <v>83</v>
+      </c>
+      <c r="E99">
+        <v>12.97</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>118</v>
+      </c>
+      <c r="B100" t="s">
+        <v>119</v>
+      </c>
+      <c r="C100">
+        <v>296</v>
+      </c>
+      <c r="D100" t="s">
+        <v>84</v>
+      </c>
+      <c r="E100">
+        <v>11.69</v>
+      </c>
+      <c r="F100">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>118</v>
+      </c>
+      <c r="B101" t="s">
+        <v>119</v>
+      </c>
+      <c r="C101">
+        <v>296</v>
+      </c>
+      <c r="D101" t="s">
+        <v>85</v>
+      </c>
+      <c r="E101">
+        <v>14.05</v>
+      </c>
+      <c r="F101">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>118</v>
+      </c>
+      <c r="B102" t="s">
+        <v>119</v>
+      </c>
+      <c r="C102">
+        <v>296</v>
+      </c>
+      <c r="D102" t="s">
+        <v>86</v>
+      </c>
+      <c r="E102">
+        <v>0.78</v>
+      </c>
+      <c r="F102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>118</v>
+      </c>
+      <c r="B103" t="s">
+        <v>119</v>
+      </c>
+      <c r="C103">
+        <v>296</v>
+      </c>
+      <c r="D103" t="s">
+        <v>87</v>
+      </c>
+      <c r="E103">
+        <v>55.93</v>
+      </c>
+      <c r="F103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>120</v>
+      </c>
+      <c r="B104" t="s">
+        <v>121</v>
+      </c>
+      <c r="D104" t="s">
+        <v>82</v>
+      </c>
+      <c r="E104">
+        <v>98.97</v>
+      </c>
+      <c r="F104">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>120</v>
+      </c>
+      <c r="B105" t="s">
+        <v>121</v>
+      </c>
+      <c r="D105" t="s">
+        <v>83</v>
+      </c>
+      <c r="E105">
+        <v>51.88</v>
+      </c>
+      <c r="F105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>120</v>
+      </c>
+      <c r="B106" t="s">
+        <v>121</v>
+      </c>
+      <c r="D106" t="s">
+        <v>84</v>
+      </c>
+      <c r="E106">
+        <v>34.2</v>
+      </c>
+      <c r="F106">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>120</v>
+      </c>
+      <c r="B107" t="s">
+        <v>121</v>
+      </c>
+      <c r="D107" t="s">
+        <v>85</v>
+      </c>
+      <c r="E107">
+        <v>33.63</v>
+      </c>
+      <c r="F107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>120</v>
+      </c>
+      <c r="B108" t="s">
+        <v>121</v>
+      </c>
+      <c r="D108" t="s">
+        <v>86</v>
+      </c>
+      <c r="E108">
+        <v>3.13</v>
+      </c>
+      <c r="F108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>120</v>
+      </c>
+      <c r="B109" t="s">
+        <v>121</v>
+      </c>
+      <c r="D109" t="s">
+        <v>87</v>
+      </c>
+      <c r="E109">
+        <v>55.93</v>
+      </c>
+      <c r="F109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>122</v>
+      </c>
+      <c r="B110" t="s">
+        <v>123</v>
+      </c>
+      <c r="D110" t="s">
+        <v>82</v>
+      </c>
+      <c r="E110">
+        <v>66.93</v>
+      </c>
+      <c r="F110">
+        <v>79.42</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>122</v>
+      </c>
+      <c r="B111" t="s">
+        <v>123</v>
+      </c>
+      <c r="D111" t="s">
+        <v>83</v>
+      </c>
+      <c r="E111">
+        <v>0</v>
+      </c>
+      <c r="F111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>122</v>
+      </c>
+      <c r="B112" t="s">
+        <v>123</v>
+      </c>
+      <c r="D112" t="s">
+        <v>84</v>
+      </c>
+      <c r="E112">
+        <v>0</v>
+      </c>
+      <c r="F112">
+        <v>2.92</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>122</v>
+      </c>
+      <c r="B113" t="s">
+        <v>123</v>
+      </c>
+      <c r="D113" t="s">
+        <v>85</v>
+      </c>
+      <c r="E113">
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>2.43</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>122</v>
+      </c>
+      <c r="B114" t="s">
+        <v>123</v>
+      </c>
+      <c r="D114" t="s">
+        <v>86</v>
+      </c>
+      <c r="E114">
+        <v>0</v>
+      </c>
+      <c r="F114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>122</v>
+      </c>
+      <c r="B115" t="s">
+        <v>123</v>
+      </c>
+      <c r="D115" t="s">
+        <v>87</v>
+      </c>
+      <c r="E115">
+        <v>55.93</v>
+      </c>
+      <c r="F115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>124</v>
+      </c>
+      <c r="B116" t="s">
+        <v>125</v>
+      </c>
+      <c r="D116" t="s">
+        <v>82</v>
+      </c>
+      <c r="E116">
+        <v>93.01</v>
+      </c>
+      <c r="F116">
+        <v>81.03</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>124</v>
+      </c>
+      <c r="B117" t="s">
+        <v>125</v>
+      </c>
+      <c r="D117" t="s">
+        <v>83</v>
+      </c>
+      <c r="E117">
+        <v>0</v>
+      </c>
+      <c r="F117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>124</v>
+      </c>
+      <c r="B118" t="s">
+        <v>125</v>
+      </c>
+      <c r="D118" t="s">
+        <v>84</v>
+      </c>
+      <c r="E118">
+        <v>12.28</v>
+      </c>
+      <c r="F118">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>124</v>
+      </c>
+      <c r="B119" t="s">
+        <v>125</v>
+      </c>
+      <c r="D119" t="s">
+        <v>85</v>
+      </c>
+      <c r="E119">
+        <v>22.58</v>
+      </c>
+      <c r="F119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>124</v>
+      </c>
+      <c r="B120" t="s">
+        <v>125</v>
+      </c>
+      <c r="D120" t="s">
+        <v>86</v>
+      </c>
+      <c r="E120">
+        <v>0</v>
+      </c>
+      <c r="F120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>124</v>
+      </c>
+      <c r="B121" t="s">
+        <v>125</v>
+      </c>
+      <c r="D121" t="s">
+        <v>87</v>
+      </c>
+      <c r="E121">
+        <v>55.93</v>
+      </c>
+      <c r="F121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>126</v>
+      </c>
+      <c r="B122" t="s">
+        <v>127</v>
+      </c>
+      <c r="D122" t="s">
+        <v>82</v>
+      </c>
+      <c r="E122">
+        <v>77.93</v>
+      </c>
+      <c r="F122">
+        <v>80.45</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>126</v>
+      </c>
+      <c r="B123" t="s">
+        <v>127</v>
+      </c>
+      <c r="D123" t="s">
+        <v>83</v>
+      </c>
+      <c r="E123">
+        <v>0</v>
+      </c>
+      <c r="F123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>126</v>
+      </c>
+      <c r="B124" t="s">
+        <v>127</v>
+      </c>
+      <c r="D124" t="s">
+        <v>84</v>
+      </c>
+      <c r="E124">
+        <v>0.28</v>
+      </c>
+      <c r="F124">
+        <v>2.38</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>126</v>
+      </c>
+      <c r="B125" t="s">
+        <v>127</v>
+      </c>
+      <c r="D125" t="s">
+        <v>85</v>
+      </c>
+      <c r="E125">
+        <v>0</v>
+      </c>
+      <c r="F125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>126</v>
+      </c>
+      <c r="B126" t="s">
+        <v>127</v>
+      </c>
+      <c r="D126" t="s">
+        <v>86</v>
+      </c>
+      <c r="E126">
+        <v>0</v>
+      </c>
+      <c r="F126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
+        <v>127</v>
+      </c>
+      <c r="D127" t="s">
+        <v>87</v>
+      </c>
+      <c r="E127">
+        <v>55.93</v>
+      </c>
+      <c r="F127">
         <v>0</v>
       </c>
     </row>
@@ -2256,7 +4258,7 @@
         <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>96</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2286,7 +4288,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>129</v>
       </c>
       <c r="B2">
         <v>44.64</v>
@@ -2297,7 +4299,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="B3">
         <v>41.2</v>
@@ -2308,7 +4310,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>131</v>
       </c>
       <c r="B4">
         <v>52.54</v>
@@ -2319,7 +4321,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="B5">
         <v>69.53</v>
@@ -2336,218 +4338,639 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="8" width="22" customWidth="1"/>
+    <col min="1" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B2">
-        <v>54.86</v>
-      </c>
-      <c r="C2">
-        <v>31.52</v>
-      </c>
-      <c r="D2" t="s">
-        <v>108</v>
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D2">
+        <v>44.64</v>
       </c>
       <c r="E2">
-        <v>26.05</v>
-      </c>
-      <c r="F2">
-        <v>-19.47</v>
-      </c>
-      <c r="G2">
-        <v>-20.71</v>
-      </c>
-      <c r="H2">
-        <v>-23.34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12.59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3">
-        <v>55.64</v>
-      </c>
-      <c r="C3">
-        <v>40.9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>108</v>
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3">
+        <v>41.2</v>
       </c>
       <c r="E3">
-        <v>35.24</v>
-      </c>
-      <c r="F3">
-        <v>-10.65</v>
-      </c>
-      <c r="G3">
-        <v>-12.4</v>
-      </c>
-      <c r="H3">
-        <v>-14.74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>13.34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B4">
-        <v>70.76</v>
-      </c>
-      <c r="C4">
-        <v>52.92</v>
-      </c>
-      <c r="D4" t="s">
-        <v>110</v>
+        <v>38</v>
+      </c>
+      <c r="B4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4">
+        <v>52.54</v>
       </c>
       <c r="E4">
-        <v>48.13</v>
-      </c>
-      <c r="F4">
-        <v>-12.25</v>
-      </c>
-      <c r="G4">
-        <v>-14.67</v>
-      </c>
-      <c r="H4">
-        <v>-17.84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12.44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5">
-        <v>62.04</v>
-      </c>
-      <c r="C5">
-        <v>42.49</v>
-      </c>
-      <c r="D5" t="s">
-        <v>111</v>
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D5">
+        <v>69.53</v>
       </c>
       <c r="E5">
-        <v>38.28</v>
-      </c>
-      <c r="F5">
-        <v>-15.03</v>
-      </c>
-      <c r="G5">
-        <v>-17.2</v>
-      </c>
-      <c r="H5">
-        <v>-19.55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>11.21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B6">
-        <v>44.69</v>
-      </c>
-      <c r="C6">
-        <v>33.07</v>
-      </c>
-      <c r="D6" t="s">
-        <v>112</v>
+        <v>134</v>
+      </c>
+      <c r="B6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D6">
+        <v>40</v>
       </c>
       <c r="E6">
-        <v>25.81</v>
-      </c>
-      <c r="F6">
-        <v>-7.76</v>
-      </c>
-      <c r="G6">
-        <v>-9.25</v>
-      </c>
-      <c r="H6">
-        <v>-11.89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19.37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>95</v>
-      </c>
-      <c r="B7">
-        <v>45.56</v>
-      </c>
-      <c r="C7">
-        <v>35.18</v>
-      </c>
-      <c r="D7" t="s">
-        <v>108</v>
+        <v>134</v>
+      </c>
+      <c r="B7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D7">
+        <v>16.94</v>
       </c>
       <c r="E7">
-        <v>28.76</v>
-      </c>
-      <c r="F7">
-        <v>-7.78</v>
-      </c>
-      <c r="G7">
-        <v>-8.77</v>
-      </c>
-      <c r="H7">
-        <v>-10.38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8">
-        <v>53.24</v>
-      </c>
-      <c r="C8">
-        <v>12.31</v>
-      </c>
-      <c r="D8" t="s">
-        <v>108</v>
+        <v>134</v>
+      </c>
+      <c r="B8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>7.25</v>
-      </c>
-      <c r="F8">
-        <v>-37.51</v>
-      </c>
-      <c r="G8">
-        <v>-37.71</v>
-      </c>
-      <c r="H8">
-        <v>-40.93</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" t="s">
+        <v>140</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12">
+        <v>6.03</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D13">
+        <v>78.04</v>
+      </c>
+      <c r="E13">
+        <v>19.24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14">
+        <v>59.43</v>
+      </c>
+      <c r="E14">
+        <v>14.73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>143</v>
+      </c>
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D15">
+        <v>16.64</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" t="s">
+        <v>138</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>143</v>
+      </c>
+      <c r="B18" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" t="s">
+        <v>140</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>143</v>
+      </c>
+      <c r="B20" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" t="s">
+        <v>141</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>143</v>
+      </c>
+      <c r="B21" t="s">
+        <v>130</v>
+      </c>
+      <c r="C21" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21">
+        <v>54.51</v>
+      </c>
+      <c r="E21">
+        <v>25.49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>144</v>
+      </c>
+      <c r="B22" t="s">
+        <v>131</v>
+      </c>
+      <c r="C22" t="s">
+        <v>135</v>
+      </c>
+      <c r="D22">
+        <v>57.09</v>
+      </c>
+      <c r="E22">
+        <v>19.32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>144</v>
+      </c>
+      <c r="B23" t="s">
+        <v>131</v>
+      </c>
+      <c r="C23" t="s">
+        <v>136</v>
+      </c>
+      <c r="D23">
+        <v>32.36</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>144</v>
+      </c>
+      <c r="B24" t="s">
+        <v>131</v>
+      </c>
+      <c r="C24" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>144</v>
+      </c>
+      <c r="B25" t="s">
+        <v>131</v>
+      </c>
+      <c r="C25" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>144</v>
+      </c>
+      <c r="B26" t="s">
+        <v>131</v>
+      </c>
+      <c r="C26" t="s">
+        <v>139</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>144</v>
+      </c>
+      <c r="B27" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" t="s">
+        <v>140</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>144</v>
+      </c>
+      <c r="B28" t="s">
+        <v>131</v>
+      </c>
+      <c r="C28" t="s">
+        <v>141</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29" t="s">
+        <v>142</v>
+      </c>
+      <c r="D29">
+        <v>82.34</v>
+      </c>
+      <c r="E29">
+        <v>16.85</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B30" t="s">
+        <v>132</v>
+      </c>
+      <c r="C30" t="s">
+        <v>135</v>
+      </c>
+      <c r="D30">
+        <v>86.93</v>
+      </c>
+      <c r="E30">
+        <v>17.28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>145</v>
+      </c>
+      <c r="B31" t="s">
+        <v>132</v>
+      </c>
+      <c r="C31" t="s">
+        <v>136</v>
+      </c>
+      <c r="D31">
+        <v>67.66</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>145</v>
+      </c>
+      <c r="B32" t="s">
+        <v>132</v>
+      </c>
+      <c r="C32" t="s">
+        <v>137</v>
+      </c>
+      <c r="D32">
+        <v>8.77</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>145</v>
+      </c>
+      <c r="B33" t="s">
+        <v>132</v>
+      </c>
+      <c r="C33" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>145</v>
+      </c>
+      <c r="B34" t="s">
+        <v>132</v>
+      </c>
+      <c r="C34" t="s">
+        <v>139</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>145</v>
+      </c>
+      <c r="B35" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" t="s">
+        <v>140</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>145</v>
+      </c>
+      <c r="B36" t="s">
+        <v>132</v>
+      </c>
+      <c r="C36" t="s">
+        <v>141</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" t="s">
+        <v>132</v>
+      </c>
+      <c r="C37" t="s">
+        <v>142</v>
+      </c>
+      <c r="D37">
+        <v>89.13</v>
+      </c>
+      <c r="E37">
+        <v>15.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Collapsible sections, regrouped insights, text/heading refinements
- Make every section a collapsible dropdown (click heading to
  minimize/expand; PDF export expands all sections first, then restores)
- Bold sentence-case section headings; update heading texts per request
- Remove the Həftəlik tempo dashboard; keep weekly-change analysis only
- Add a passive-voice "?" explanation to the Plana uyğunluq indicator
  and a single brief velocity summary note
- Regroup insights into concise bullet blocks: "Tikinti gedişatında
  müəyyən olunan problemlər" and "İcra gedişatındakı irəliləyiş";
  drop the workforce-pending insight; trim analiz to first sentence
- KPI subtitle "Məlumat əlavə edilməyib"; Hazırlanma tarixi 17.06.2026

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QYNS9XGzgg9T4WgeLa9vfk
</commit_message>
<xml_diff>
--- a/cities/qervend/source.xlsx
+++ b/cities/qervend/source.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="192">
   <si>
     <t>Sahə</t>
   </si>
@@ -34,7 +34,7 @@
     <t>projectTitle</t>
   </si>
   <si>
-    <t>QƏRVƏND KƏNDİ — TİKİNTİ GEDİŞATI HESABATI</t>
+    <t>Qərvənd kəndi üzrə tikinti gedişatı hesabatı</t>
   </si>
   <si>
     <t>village</t>
@@ -178,7 +178,7 @@
     <t>İŞÇİ SAYI (GÜNDƏLİK)</t>
   </si>
   <si>
-    <t>Gündəlik hesabat daxil edilməyib</t>
+    <t>Məlumat əlavə edilməyib</t>
   </si>
   <si>
     <t>violet</t>
@@ -571,7 +571,7 @@
     <t>velPoint1</t>
   </si>
   <si>
-    <t>Keçən ay (≈28.05)</t>
+    <t>28.05</t>
   </si>
   <si>
     <t>velPoint2</t>
@@ -596,9 +596,6 @@
   </si>
   <si>
     <t>workforceEmptyNote</t>
-  </si>
-  <si>
-    <t>İşçi heyəti və texnika üzrə gündəlik hesabat hələ bu hesabata əlavə edilməyib. Məlumat Excel-ə əlavə edilib göndərildikdə bu bölmə avtomatik olaraq qrafikləri göstərəcək.</t>
   </si>
   <si>
     <t>workforceAlert</t>
@@ -1553,12 +1550,12 @@
         <v>190</v>
       </c>
       <c r="B17" t="s">
-        <v>191</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>

</xml_diff>